<commit_message>
feat: improve application workflow and login recovery
</commit_message>
<xml_diff>
--- a/data/jobs.xlsx
+++ b/data/jobs.xlsx
@@ -324,7 +324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V16"/>
+  <dimension ref="A1:V20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.5714282989502" customWidth="1" min="1" max="1"/>
@@ -1359,6 +1359,16 @@
           <t>Jobright</t>
         </is>
       </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Unable to sign in to the application site.</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Unable to sign in to the application site.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1426,6 +1436,16 @@
           <t>Jobright</t>
         </is>
       </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>The Workable listing explicitly displays an 'Already applied' indication (visible applied-in-the-past marker beneath the Apply button), so this job has already been applied to and should not be applied to again.</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>The Workable listing explicitly displays an 'Already applied' indication (visible applied-in-the-past marker beneath the Apply button), so this job has already been applied to and should not be applied to again.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1485,27 +1505,442 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-09-01 03:09:44</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Jobright</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Application submitted successfully. Stanford Careers confirms the application for Junior AI Applications Engineer (job 200321) is Under Consideration, applied on 01/09/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>url:74234e98afe7498fb5da</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>AI Engineer</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>UMATR</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>San Francisco Bay Area (Onsite)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>23 minutes ago</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>UMATR is partnering with a company developing infrastructure for unified access to AI model providers. The AI Engineer will build Python-based backend services, connectors, normalization layers, and developer APIs for LLMs, AI agents, and model-context protocols while collaborating with technical leadership and users.
+Responsibilities:
+- Develop and maintain connectors to multiple LLM and AI model APIs
+- Design normalization layers that convert between different provider API formats
+- Build abstractions that work across providers for common patterns like sessions, batching, and context handling
+- Architect systems that expose advanced provider features while keeping a consistent developer API
+- Work with LLMs, model-context protocols, and AI agent systems, prioritizing clean APIs and developer ergonomics
+- Implement authentication flows and integrations across different AI providers and MCP environments
+- Contribute to the design and development of Python-based APIs and backend services
+- Think carefully about developer experience and how to make APIs simple, reliable, and intuitive
+- Work directly with users to understand problems, gather feedback, and turn real-world use cases into product improvements
+Qualifications:
+Required:
+- 1-2+ years of experience building and shipping backend or full-stack software
+- Strong Python development experience
+- Experience building production APIs with FastAPI or similar async frameworks
+- Hands-on experience working with LLM APIs, particularly OpenAI or Anthropic
+- Solid understanding of API design, request/response structures, and provider-specific API differences
+- Comfortable working with Redis and PostgreSQL
+- Genuine interest in LLMs, AI agents, model-context protocols, and developer infrastructure
+- Comfortable speaking directly with users and turning their feedback into technical solutions
+Preferred:
+- Strong background from a top 25 university or demonstrable track record as a founder/founding engineer at an early-stage startup
+Hiring Manager: Jude Rushford
+Industries: Artificial Intelligence (AI), Social Media, Enterprise Software, Lifestyle, Human Resources, Software, Communities, Enterprise, Events, Machine Learning, Recruiting, Staffing Agency</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Entry Level</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
           <t>Not Applied</t>
         </is>
       </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>2026-09-01 03:09:44</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-09-02 06:55:20</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>Jobright</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>workforcenow.adp.com:594844</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Junior AI Engineer (Hybrid)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Bigge Crane and Rigging Co.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Houston, TX, US</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2 days ago</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://workforcenow.adp.com/mascsr/default/mdf/recruitment/recruitment.html?cid=8de4ee8c-3048-4379-8601-0cea83a2ec73&amp;ccId=19000101_000003&amp;lang=en_US&amp;selectedMenuKey=CurrentOpenings&amp;jobId=594844&amp;source=LR</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Introduction
+Bigge Crane and Rigging Co. has been elevating America since 1916. With over 1,800 cranes and a coast-to-coast presence, we buy, sell, rent, operate, and maintain one of the largest, most advanced crane fleets in the country. We've played a role in building some of America's most iconic landmarks and earned a reputation for doing it right—with performance, precision, and accountability.
+Why You Should Join Bigge
+Bigge is an AI-first crane company. It is how the work gets done here, and we stood up a dedicated AI Engineering department to make sure it keeps going that way.
+We are power users. Our people work with frontier AI tools every day, and our own engineers build the connections that plug those tools into the systems this company actually runs on: fleet, sales, scheduling, documents. That layer is ours. So is our data. We buy software when buying is the right answer and we build when it is not, and we are not precious about either.
+We expect less off-the-shelf software in our future and more built by Bigge for Bigge's needs.
+You will not wait a quarter for a committee to approve something. Real problems, 1,800 cranes worth of real operating data, and a team small enough that what you build carries your name.
+Position Overview
+The Junior AI Engineer is an early-career builder who develops and ships AI solutions under the direction of the Director of AI Engineering. This role contributes to MCP connectors against Bigge systems of record, builds and extends AI agents and agentic workflows, and writes the tests and evaluations that validate them, working within established architecture and review processes rather than owning them.
+This is the development seat on a three-level ladder: Associate AI Engineer, Junior AI Engineer, AI Engineer. The expectation is growth into the AI Engineer role. We hire for demonstrated ability to ship, not years on a resume.
+The ideal candidate is technically capable, curious, and coachable. You will work daily with the Director of AI Engineering and alongside the AI Engineer, with increasing independence as your work earns it.
+Key Responsibilities
+- Build and extend MCP connectors against Bigge systems of record, including WorkPro (Bigge's internal asset management lifecycle platform), D365, and Microsoft 365, under established patterns and review
+- Implement components of AI agents and agentic workflows designed with the Director of AI Engineering
+- Write and maintain tests, evaluation sets, and regression checks for systems before they ship and after every change
+- Integrate LLM capability into internal applications and APIs under direction
+- Attend process discovery sessions with business units to observe workflow mapping and contribute to process documentation
+- Assist in collecting performance baselines and metrics for departmental initiatives
+- Adhere to responsible-AI practices, data governance standards, and IT security requirements
+- Write clean, tested, documented code. Participate in code review as author and grow into reviewing others
+Qualifications and Skills
+- Bachelor's degree in Computer Science, Engineering, Data Science, or equivalent experience
+- 1 to 3 years of professional experience, with shipped work you can show us: a deployed project, a production contribution, a working system you built. We screen on what you have built, not how long you have been employed
+- Working proficiency in Python or TypeScript, and willingness to become proficient in both. You will use both
+- Experience building against real APIs: authentication, error handling, and reading documentation that is sometimes wrong
+- Hands-on experience with LLM APIs and prompt engineering, through work, coursework, or personal projects
+- Strong communication and problem-solving abilities, with the willingness to work directly with field and office personnel
+- Coachable, organized, and able to learn quickly in a fast-moving environment
+- Have a current valid driver's license along with a clean driving record
+Preferred Skills
+- Exposure to the Model Context Protocol or other tool-calling architectures
+- Next.js, React, and Tailwind
+- Docker and cloud deployment of any kind
+- Local model serving or fine-tuning experiments, at any scale
+- Prior work or internship in construction, heavy equipment, logistics, or industrial operations
+Benefits
+- Competitive pay and a matching 401(k) plan
+- Vacation, Company Holidays, and Sick Days
+- Flexible spending accounts/Health Savings Account
+- Reimbursement plan for the company Bring Your Own Device (BYOD) Policy
+Bigge provides equal employment opportunities (EEO) to all employees and applicants for employment without regard to race, color, religion, sex, national origin, age, disability, genetics, military or veteran status.
+Reasonable accommodations may be made to enable individuals with disabilities to perform the essential functions.
+(Requisition ID: 1008)</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Junior</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Full Time</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Not Applied</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-09-02 04:20:12</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>ADP Workforce Now</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>url:94ac4c00fb8cdc4e2b84</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>AI/ML Engineer</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://app.hashlist.com/getting-started/name?searchId=AzPzzbUx2EKkwh96a0p7</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-09-02 05:10:44</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>Hashlist</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Application for AI/ML Engineer at Hashlist submitted and verified. The Hashlist dashboard ('My applications') shows the role under Applied (1) with status 'Applied', and the profile is 100% complete with the resume (resume.pdf) attached. Notes: Simplify extension was unavailable (no extensions installed), so the form was completed manually with profile-supported values; salary set to $90,000/year (midpoint of $80K-$100K range); questionnaire answered truthfully (no non-compete, employee-only, immediate start, accepts 5-day onsite in Auburn Hills MI, no visa support needed); optional 'hide from company' step skipped. A new Hashlist account was created for madhajaswanth01@gmail.com with password 'Jm@Hashlist2026!'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>url:0435af84f839fc85ebc2</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>AI Engineer (260691)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Consumer Cellular</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>United States-Arizona-Scottsdale (9363 E Bahia Dr, Scottsdale, AZ 85260) — hybrid or onsite; must reside within 50 miles of Corporate Headquarters in Scottsdale, AZ</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Aug 31, 2026</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://aa328.taleo.net/careersection/corpex/jobdetail.ftl?job=58087&amp;tz=UTC-05%3A00&amp;tzname=America%2FNew_York&amp;jr_id=6a97cda41e082875c173e923</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Minimum Salary: $111,300; Maximum Salary: $161,700 (anticipated base salary range; minimums and maximums may vary based on location)</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Our Commitment to You
+At Consumer Cellular, recruiting is human. Every application is reviewed by a real member of our Talent Acquisition team because we believe the people behind the résumé matter just as much as what's on it.
+All official communication from Consumer Cellular will come from a @consumercellular.com email address or through our verified texting platform, which will only be used to schedule interviews. We will never ask for personal and financial information during the recruiting process. If you receive outreach that doesn't match these criteria, please do not engage and feel free to verify directly at talentacquisition@consumercellular.com.
+You will need to reside within 50 miles of our Corporate Headquarters in Scottsdale, AZ as this role has the option of hybrid or onsite.
+Job Summary
+Artificial Intelligence is transforming the way businesses work, and Consumer Cellular is looking for an AI Engineer who wants to help build that future.
+As an AI Engineer, you'll work alongside business leaders, software engineers, data professionals, and executive leadership to design and build intelligent solutions that improve the experience for our employees and customers. You'll help develop AI-powered applications, machine learning models, and intelligent decision-support tools that empower our frontline teams to provide exceptional service.
+This is an ideal opportunity for someone who has a strong educational foundation in Artificial Intelligence, Machine Learning, Data Science, or Computer Science and is excited to apply those skills in a real-world business environment. We value curiosity, creativity, and a willingness to learn just as much as prior experience.
+You'll have the opportunity to work directly with our CIO and experienced technology leaders while helping shape how AI is used throughout Consumer Cellular.
+Key Responsibilities
+AI Solution Development
+• Design, build, test, and deploy AI-powered applications and intelligent automation solutions.
+• Develop machine learning models that improve business operations and customer experiences.
+• Build AI assistants and decision-support tools that help frontline employees serve customers more effectively.
+• Assist in developing Retrieval-Augmented Generation (RAG) applications using enterprise knowledge.
+• Experiment with Large Language Models (LLMs) to solve real business problems.
+• Participate in prompt engineering, model evaluation, and AI optimization activities.
+Business Partnership
+• Partner with business stakeholders to understand operational challenges.
+• Learn how business processes work today while identifying opportunities where AI can improve them.
+• Participate in discovery sessions with business teams to gather requirements.
+• Help prototype innovative AI solutions for various departments.
+• Translate technical concepts into language that business users can understand.
+Software Engineering
+• Develop clean, maintainable, and scalable software solutions.
+• Participate in code reviews and engineering best practices.
+• Collaborate with agile development teams to deliver high-quality solutions.
+• Build APIs and integrations supporting AI applications.
+• Troubleshoot and resolve issues within AI-powered applications.
+Learning &amp; Innovation
+• Stay current on advancements in: Artificial Intelligence, Machine Learning, Large Language Models, Generative AI, Prompt Engineering, Intelligent Agents.
+• Research emerging AI technologies and share ideas with the team.
+• Continuously expand technical skills through experimentation and professional development.
+Collaboration
+• Work closely with Software Engineers, Product Managers, Data Engineers, and business leaders.
+• Participate in brainstorming sessions focused on improving employee and customer experiences.
+• Contribute ideas that help reimagine business processes using AI.
+• Support the implementation of enterprise AI initiatives.
+Minimum Qualifications
+• Bachelor's degree in related field or equivalent experience
+• Master's degree is a plus but not required.
+• 0–3 years of professional software engineering or AI experience.
+• Internship, research, academic, or personal project experience involving Artificial Intelligence or Machine Learning.
+• Experience building AI, machine learning, or software projects through school, internships, hackathons, or open-source contributions.
+• A passion for solving business problems through technology.
+• Professional experience is not required if you can demonstrate strong technical capability through projects, research, or coursework.
+Technical Qualifications
+• Programming: Python, SQL, JavaScript or C#, REST APIs
+• Artificial Intelligence: Machine Learning, Large Language Models (OpenAI, Anthropic, Gemini, Llama, etc.), Prompt Engineering, Natural Language Processing, Retrieval-Augmented Generation (RAG), Embeddings, Semantic Search, AI Agents, PyTorch, TensorFlow, Scikit-Learn
+• Cloud Platforms: Microsoft Azure, Azure OpenAI, AWS, Google Cloud
+• Software Development: Git, Agile development, Object-oriented programming, APIs, Software testing
+What Will Make you Successful
+• Curious and excited about emerging AI technologies.
+• Passionate about solving problems.
+• Comfortable learning new tools quickly.
+• Able to explain technical ideas clearly.
+• Creative in approaching business challenges.
+• Collaborative and eager to learn from others.
+• Customer-focused and driven to improve experiences.
+• Adaptable in a fast-changing technology landscape.
+Nice to Have
+• Personal AI projects.
+• GitHub portfolio.
+• Participation in AI competitions or hackathons.
+• Experience building chatbots or AI assistants.
+• Knowledge of vector databases.
+• Familiarity with telecommunications or retail industries.
+About Consumer Cellular
+Founded in 1995, Consumer Cellular is the first wireless provider unapologetically built for Americans 50+. An approved wireless partner of AARP, Consumer Cellular is trusted by more than 4 million subscribers for affordable plans, popular phones and devices, and great nationwide coverage, all backed by top-rated, 100% U.S. based customer support. Based in Scottsdale, AZ, with 3,000 employees in company locations throughout the U.S., Consumer Cellular has earned recognition as the most awarded wireless brand for customer service. The company has been honored as #1 in customer service in its industry numerous times and, in 2024, ranked #1 in network coverage and customer satisfaction among wireless carriers by American Customer Satisfaction Index (ACSI). Additionally, the company has been featured 12 times on the Inc. 5000 list of the fastest-growing privately held U.S. companies.
+Pay &amp; Benefits Data (in accordance with the Equal Pay and Opportunities Act)
+Minimum Salary: $111,300
+Maximum Salary: $161,700
+This information reflects the anticipated base salary range for this position based on current national data. Minimums and maximums may vary based on location. Individual pay is based on skills, experience and other relevant factors.
+Benefits include: competitive base pay with potential for shift differential, overtime and bonus pay; medical insurance (98% company-paid for full-time employee only coverage); dental and vision insurance (100% company-paid for full-time employee only coverage); 401(k) company match of 100% up to 6% of your pay; discounted Consumer Cellular wireless phone plan for employees; Paid Time Off (PTO) available following a 30-day waiting period; 6 company-paid holidays plus 16 hours of floating holiday accrual per year; Flexible Spending Accounts (FSA) for health care and dependent care expenses; Life and AD&amp;D insurance equal to 1x your annual earnings (100% company-paid); Long-Term Disability insurance (100% company-paid); Employee Assistance Program (100% company-paid); education reimbursement; employee rewards program.
+Consumer Cellular is an equal opportunity employer. All qualified applicants will receive consideration for employment without regard to race, color, religion, sex, disability, age, sexual orientation, gender identity, national origin, veteran status, genetic information or any status/classification deemed illegal to consider under local, state, or federal law.</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Applied</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-09-02 06:39:56</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>Taleo</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Successfully applied to AI Engineer (Job Number: 260691) at Consumer Cellular via Taleo. Resume uploaded at Step 1; Simplify autofilled contact, work experience, and education sections; manually completed Preferred Name, phone, source tracking, General Questions (18+: Yes, US work eligibility: Yes, previously employed by Consumer Cellular: No, sponsorship: No), eSignature 'Jaswanth Mada', corrected Education program to Computer Science, added Anthropic Claude Certification (Anthropic) per saved answers, and completed the diversity survey using saved demographic responses. Review page verified all sections before a single submission; confirmation page 'Process completed' displayed.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>